<commit_message>
space heating, dhw and electrical curve plotting
</commit_message>
<xml_diff>
--- a/pycity_calc/toolbox/mc_helpers/Morris_analysis/City_generation/Morris_values.xlsx
+++ b/pycity_calc/toolbox/mc_helpers/Morris_analysis/City_generation/Morris_values.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="118">
   <si>
     <t>longitude</t>
   </si>
@@ -370,6 +370,9 @@
   </si>
   <si>
     <t>6.001</t>
+  </si>
+  <si>
+    <t>1977</t>
   </si>
 </sst>
 </file>
@@ -794,8 +797,8 @@
       <c r="A8" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="1">
-        <v>1970</v>
+      <c r="B8" s="1" t="s">
+        <v>117</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>114</v>
@@ -875,7 +878,7 @@
         <v>21</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
dhw rescaling and Salib deletion
</commit_message>
<xml_diff>
--- a/pycity_calc/toolbox/mc_helpers/Morris_analysis/City_generation/Morris_values.xlsx
+++ b/pycity_calc/toolbox/mc_helpers/Morris_analysis/City_generation/Morris_values.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="120">
   <si>
     <t>longitude</t>
   </si>
@@ -117,9 +117,6 @@
     <t>0.9</t>
   </si>
   <si>
-    <t>0.15</t>
-  </si>
-  <si>
     <t>0.25</t>
   </si>
   <si>
@@ -327,9 +324,6 @@
     <t>latitude</t>
   </si>
   <si>
-    <t>6.00</t>
-  </si>
-  <si>
     <t>263</t>
   </si>
   <si>
@@ -357,19 +351,31 @@
     <t>0.01</t>
   </si>
   <si>
-    <t>1.05</t>
-  </si>
-  <si>
     <t>1.010</t>
   </si>
   <si>
+    <t>50.775</t>
+  </si>
+  <si>
+    <t>50.776</t>
+  </si>
+  <si>
+    <t>6.083</t>
+  </si>
+  <si>
+    <t>6.084</t>
+  </si>
+  <si>
+    <t>269</t>
+  </si>
+  <si>
+    <t>0.75</t>
+  </si>
+  <si>
+    <t>0.3</t>
+  </si>
+  <si>
     <t>2015</t>
-  </si>
-  <si>
-    <t>50.001</t>
-  </si>
-  <si>
-    <t>6.001</t>
   </si>
   <si>
     <t>1977</t>
@@ -720,22 +726,22 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1">
-        <v>50</v>
+      <c r="B1" s="1" t="s">
+        <v>111</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -743,10 +749,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C3" s="1">
-        <v>268</v>
+        <v>101</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
@@ -765,10 +771,10 @@
         <v>10</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -779,7 +785,7 @@
         <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -798,10 +804,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -883,161 +889,161 @@
     </row>
     <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>33</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>31</v>
@@ -1048,29 +1054,29 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B31" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>17</v>
@@ -1081,10 +1087,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>25</v>
@@ -1092,21 +1098,21 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>17</v>
@@ -1114,222 +1120,222 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C41" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B42" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C42" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B43" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B52" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C52" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="C52" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B53" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C53" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>